<commit_message>
feat(leadnet): add database reactivation and angi/lsa features to capture page
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sales/LeadNet_Verified_DBPR_Hitlist.xlsx
+++ b/sales/LeadNet_Verified_DBPR_Hitlist.xlsx
@@ -1,15 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J-SHMONEY\Desktop\Intent\sales\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6627F546-62A8-4876-88FD-61C4CA6A0D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hitlist Pipeline" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -754,8 +773,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -985,15 +1004,6 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1012,19 +1022,36 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1062,7 +1089,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1096,6 +1123,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1130,9 +1158,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1305,1224 +1334,1224 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" customWidth="1"/>
+    <col min="4" max="4" width="35.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="6" max="6" width="61.28515625" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" customWidth="1"/>
     <col min="8" max="9" width="18.7109375" customWidth="1"/>
     <col min="10" max="10" width="26.7109375" customWidth="1"/>
     <col min="11" max="11" width="24.7109375" customWidth="1"/>
     <col min="12" max="12" width="18.7109375" customWidth="1"/>
     <col min="13" max="13" width="22.7109375" customWidth="1"/>
-    <col min="14" max="14" width="44.7109375" customWidth="1"/>
-    <col min="15" max="15" width="30.7109375" customWidth="1"/>
+    <col min="14" max="14" width="121.7109375" customWidth="1"/>
+    <col min="15" max="15" width="93.85546875" customWidth="1"/>
     <col min="16" max="16" width="24.7109375" customWidth="1"/>
     <col min="17" max="17" width="18.7109375" customWidth="1"/>
     <col min="18" max="18" width="16.7109375" customWidth="1"/>
-    <col min="19" max="19" width="38.7109375" customWidth="1"/>
+    <col min="19" max="19" width="127.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:19" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
     </row>
-    <row r="3" spans="1:19">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2" t="s">
+      <c r="F3" s="8"/>
+      <c r="G3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
+      <c r="H3" s="8"/>
+      <c r="I3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="2"/>
+      <c r="J3" s="8"/>
     </row>
-    <row r="4" spans="1:19">
-      <c r="A4" s="3">
+    <row r="4" spans="1:19" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
         <f>COUNTA(C7:C200)</f>
-        <v>0</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3">
+        <v>20</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9">
         <f>COUNTIF(B7:B200, "A*")</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3">
+        <v>11</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9">
         <f>COUNTIF(A7:A200, "Demo Booked")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3">
+      <c r="F4" s="9"/>
+      <c r="G4" s="9">
         <f>COUNTIF(A7:A200, "&lt;&gt;Not Contacted") - COUNTBLANK(A7:A200)</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3">
+        <v>3</v>
+      </c>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9">
         <f>COUNTIF(A7:A200, "Gatekeeper*") + COUNTIF(A7:A200, "Follow-up")</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="J4" s="9"/>
     </row>
-    <row r="6" spans="1:19" ht="28" customHeight="1">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="N6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="O6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="P6" s="4" t="s">
+      <c r="P6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="Q6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="R6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="S6" s="4" t="s">
+      <c r="S6" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="22" customHeight="1">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5" t="s">
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="S7" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="22" customHeight="1">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="7" t="s">
+      <c r="L8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="M8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="N8" s="7" t="s">
+      <c r="N8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="O8" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7" t="s">
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="S8" s="7" t="s">
+      <c r="S8" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="22" customHeight="1">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="L9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="M9" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="N9" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5" t="s">
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="S9" s="5" t="s">
+      <c r="S9" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="22" customHeight="1">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="7" t="s">
+      <c r="L10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M10" s="7" t="s">
+      <c r="M10" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="7" t="s">
+      <c r="N10" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="7" t="s">
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="S10" s="7" t="s">
+      <c r="S10" s="4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="22" customHeight="1">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="K11" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="L11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="M11" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="N11" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5" t="s">
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="S11" s="5" t="s">
+      <c r="S11" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="22" customHeight="1">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L12" s="7" t="s">
+      <c r="L12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M12" s="7" t="s">
+      <c r="M12" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="N12" s="7" t="s">
+      <c r="N12" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7" t="s">
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="S12" s="7" t="s">
+      <c r="S12" s="4" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="22" customHeight="1">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="K13" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="L13" s="5" t="s">
+      <c r="L13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="M13" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="N13" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5" t="s">
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="S13" s="5" t="s">
+      <c r="S13" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="22" customHeight="1">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="L14" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="M14" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="N14" s="7" t="s">
+      <c r="N14" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7" t="s">
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="S14" s="7" t="s">
+      <c r="S14" s="4" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="22" customHeight="1">
-      <c r="A15" s="8" t="s">
+    <row r="15" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="K15" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="L15" s="5" t="s">
+      <c r="L15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="M15" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="N15" s="5" t="s">
+      <c r="N15" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="O15" s="5" t="s">
+      <c r="O15" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5" t="s">
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="S15" s="5" t="s">
+      <c r="S15" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="22" customHeight="1">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="J16" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="L16" s="7" t="s">
+      <c r="L16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="M16" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="N16" s="7" t="s">
+      <c r="N16" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7" t="s">
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S16" s="7" t="s">
+      <c r="S16" s="4" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="22" customHeight="1">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I17" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="J17" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="K17" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="L17" s="5" t="s">
+      <c r="L17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M17" s="5" t="s">
+      <c r="M17" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="N17" s="5" t="s">
+      <c r="N17" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-      <c r="R17" s="5" t="s">
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="S17" s="5" t="s">
+      <c r="S17" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="22" customHeight="1">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="J18" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="K18" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="L18" s="7" t="s">
+      <c r="L18" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="M18" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="N18" s="7" t="s">
+      <c r="N18" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7" t="s">
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="S18" s="7" t="s">
+      <c r="S18" s="4" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="22" customHeight="1">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="G19" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="I19" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="J19" s="5" t="s">
+      <c r="J19" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="K19" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="L19" s="5" t="s">
+      <c r="L19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M19" s="5" t="s">
+      <c r="M19" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="N19" s="5" t="s">
+      <c r="N19" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5" t="s">
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="S19" s="5" t="s">
+      <c r="S19" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="22" customHeight="1">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="J20" s="7" t="s">
+      <c r="J20" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="K20" s="7" t="s">
+      <c r="K20" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="L20" s="7" t="s">
+      <c r="L20" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M20" s="7" t="s">
+      <c r="M20" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="N20" s="7" t="s">
+      <c r="N20" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7" t="s">
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="S20" s="7" t="s">
+      <c r="S20" s="4" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="22" customHeight="1">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="G21" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="H21" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="I21" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="J21" s="5" t="s">
+      <c r="J21" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="K21" s="5" t="s">
+      <c r="K21" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="L21" s="5" t="s">
+      <c r="L21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M21" s="5" t="s">
+      <c r="M21" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="N21" s="5" t="s">
+      <c r="N21" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="5" t="s">
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="S21" s="5" t="s">
+      <c r="S21" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="22" customHeight="1">
-      <c r="A22" s="7" t="s">
+    <row r="22" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="I22" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="L22" s="7" t="s">
+      <c r="L22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M22" s="7" t="s">
+      <c r="M22" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="N22" s="7" t="s">
+      <c r="N22" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="7"/>
-      <c r="R22" s="7" t="s">
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="S22" s="7" t="s">
+      <c r="S22" s="4" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="22" customHeight="1">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="G23" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="H23" s="5" t="s">
+      <c r="H23" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="I23" s="5" t="s">
+      <c r="I23" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="J23" s="5" t="s">
+      <c r="J23" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="K23" s="5" t="s">
+      <c r="K23" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="L23" s="5" t="s">
+      <c r="L23" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M23" s="5" t="s">
+      <c r="M23" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="N23" s="5" t="s">
+      <c r="N23" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5" t="s">
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="S23" s="5" t="s">
+      <c r="S23" s="2" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="22" customHeight="1">
-      <c r="A24" s="7" t="s">
+    <row r="24" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I24" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="J24" s="7" t="s">
+      <c r="J24" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="K24" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="L24" s="7" t="s">
+      <c r="L24" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M24" s="7" t="s">
+      <c r="M24" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="N24" s="7" t="s">
+      <c r="N24" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="7" t="s">
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="S24" s="7" t="s">
+      <c r="S24" s="4" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="22" customHeight="1">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="G25" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="H25" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="I25" s="5" t="s">
+      <c r="I25" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="J25" s="5" t="s">
+      <c r="J25" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="K25" s="5" t="s">
+      <c r="K25" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="L25" s="5" t="s">
+      <c r="L25" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M25" s="5" t="s">
+      <c r="M25" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="N25" s="5" t="s">
+      <c r="N25" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5" t="s">
+      <c r="O25" s="2"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="S25" s="5" t="s">
+      <c r="S25" s="2" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="22" customHeight="1">
-      <c r="A26" s="9" t="s">
+    <row r="26" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="I26" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="J26" s="7" t="s">
+      <c r="J26" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="K26" s="7" t="s">
+      <c r="K26" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="L26" s="7" t="s">
+      <c r="L26" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M26" s="7" t="s">
+      <c r="M26" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="N26" s="7" t="s">
+      <c r="N26" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="O26" s="7" t="s">
+      <c r="O26" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="7" t="s">
+      <c r="P26" s="4"/>
+      <c r="Q26" s="4"/>
+      <c r="R26" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="S26" s="7" t="s">
+      <c r="S26" s="4" t="s">
         <v>244</v>
       </c>
     </row>
@@ -2541,37 +2570,37 @@
     <mergeCell ref="I4:J4"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A7:A200">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A7:A200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Contacted,Called - No Answer,SMS Sent,Gatekeeper / Callback,Follow-up,Demo Booked,Closed Won,Disqualified"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B200">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B200" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"A - High (Sweet Spot / Fast Conversion),B - Medium (Scale / Multi-Tech),C - Disqualified / Do Not Call"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7:L200">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7:L200" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="K7" r:id="rId1"/>
-    <hyperlink ref="K8" r:id="rId2"/>
-    <hyperlink ref="K9" r:id="rId3"/>
-    <hyperlink ref="K10" r:id="rId4"/>
-    <hyperlink ref="K11" r:id="rId5"/>
-    <hyperlink ref="K12" r:id="rId6"/>
-    <hyperlink ref="K13" r:id="rId7"/>
-    <hyperlink ref="K14" r:id="rId8"/>
-    <hyperlink ref="K15" r:id="rId9"/>
-    <hyperlink ref="K16" r:id="rId10"/>
-    <hyperlink ref="K17" r:id="rId11"/>
-    <hyperlink ref="K18" r:id="rId12"/>
-    <hyperlink ref="K19" r:id="rId13"/>
-    <hyperlink ref="K20" r:id="rId14"/>
-    <hyperlink ref="K21" r:id="rId15"/>
-    <hyperlink ref="K22" r:id="rId16"/>
-    <hyperlink ref="K23" r:id="rId17"/>
-    <hyperlink ref="K24" r:id="rId18"/>
-    <hyperlink ref="K25" r:id="rId19"/>
-    <hyperlink ref="K26" r:id="rId20"/>
+    <hyperlink ref="K7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="K8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="K9" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="K10" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="K11" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="K12" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="K13" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="K14" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="K15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="K16" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="K17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="K18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="K19" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="K20" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="K21" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="K22" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="K23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="K24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="K25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="K26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(compliance): add TCPA SMS opt-in disclosures, contact route, and verified contractor contact numbers
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sales/LeadNet_Verified_DBPR_Hitlist.xlsx
+++ b/sales/LeadNet_Verified_DBPR_Hitlist.xlsx
@@ -1,39 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J-SHMONEY\Desktop\Intent\sales\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6627F546-62A8-4876-88FD-61C4CA6A0D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Hitlist Pipeline" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="254">
   <si>
     <t>INTENT LEADNET - VERIFIED FLORIDA DBPR &amp; SUNBIZ HITLIST</t>
   </si>
@@ -131,7 +112,10 @@
     <t>CAC1824593</t>
   </si>
   <si>
-    <t>(407) 499-6574</t>
+    <t>(407) 449-7333</t>
+  </si>
+  <si>
+    <t>(407) 236-3582</t>
   </si>
   <si>
     <t>info@toptier-cooling.com</t>
@@ -170,9 +154,6 @@
     <t>(689) 331-0895</t>
   </si>
   <si>
-    <t>(407) 633-4170</t>
-  </si>
-  <si>
     <t>service@onestopairmechanical.com</t>
   </si>
   <si>
@@ -209,7 +190,7 @@
     <t>CAC1822832 / CFC1432906</t>
   </si>
   <si>
-    <t>(407) 633-5755</t>
+    <t>(407) 401-8888</t>
   </si>
   <si>
     <t>info@arcticairtemp.com</t>
@@ -239,13 +220,16 @@
     <t>CAC1819385</t>
   </si>
   <si>
-    <t>(407) 499-3806</t>
+    <t>(800) 291-0949</t>
+  </si>
+  <si>
+    <t>(407) 502-0050</t>
   </si>
   <si>
     <t>contact@ourplaceair.com</t>
   </si>
   <si>
-    <t>https://ourplaceair.com</t>
+    <t>https://callourplace.com</t>
   </si>
   <si>
     <t>4.8 (2,274 reviews)</t>
@@ -278,7 +262,7 @@
     <t>support@experthomeservice.com</t>
   </si>
   <si>
-    <t>https://experthomeservice.com</t>
+    <t>https://cool-airconditioning.com</t>
   </si>
   <si>
     <t>4.8 (604 reviews)</t>
@@ -302,10 +286,10 @@
     <t>CAC1818721</t>
   </si>
   <si>
-    <t>(561) 418-8381</t>
-  </si>
-  <si>
-    <t>contact@therightservicefl.com</t>
+    <t>(561) 814-1600</t>
+  </si>
+  <si>
+    <t>support@therightservicefl.com</t>
   </si>
   <si>
     <t>https://therightservicefl.com</t>
@@ -335,10 +319,10 @@
     <t>CAC1820119</t>
   </si>
   <si>
-    <t>(941) 529-1072</t>
-  </si>
-  <si>
-    <t>office@hurricaneairductcleaning.com</t>
+    <t>(941) 282-7797</t>
+  </si>
+  <si>
+    <t>customercare@hurricaneairductcleaning.com</t>
   </si>
   <si>
     <t>https://hurricaneairductcleaning.com</t>
@@ -365,13 +349,16 @@
     <t>CAC1819744</t>
   </si>
   <si>
-    <t>(561) 240-5273</t>
-  </si>
-  <si>
-    <t>service@airtechmechanicalfl.com</t>
-  </si>
-  <si>
-    <t>https://airtechmechanicalfl.com</t>
+    <t>(407) 874-7351</t>
+  </si>
+  <si>
+    <t>(561) 889-0755</t>
+  </si>
+  <si>
+    <t>service@myairtechmechanical.com</t>
+  </si>
+  <si>
+    <t>https://myairtechmechanical.com</t>
   </si>
   <si>
     <t>4.9 (291 reviews)</t>
@@ -401,13 +388,13 @@
     <t>CAC1817290</t>
   </si>
   <si>
-    <t>(321) 290-9840</t>
-  </si>
-  <si>
-    <t>info@rattiairandheat.com</t>
-  </si>
-  <si>
-    <t>https://rattiairandheat.com</t>
+    <t>(321) 360-2798</t>
+  </si>
+  <si>
+    <t>Office@RattiAirandHeat.com</t>
+  </si>
+  <si>
+    <t>https://www.rattiairandheat.com</t>
   </si>
   <si>
     <t>5.0 (772 reviews)</t>
@@ -434,7 +421,10 @@
     <t>CAC1819230</t>
   </si>
   <si>
-    <t>(407) 499-8730</t>
+    <t>(407) 259-4320</t>
+  </si>
+  <si>
+    <t>(844) 396-9662</t>
   </si>
   <si>
     <t>info@swiftbrothers.com</t>
@@ -500,7 +490,7 @@
     <t>CAC1821430</t>
   </si>
   <si>
-    <t>(407) 499-6275</t>
+    <t>(407) 404-4000</t>
   </si>
   <si>
     <t>info@mechanicalone.com</t>
@@ -533,13 +523,16 @@
     <t>CAC1818168</t>
   </si>
   <si>
-    <t>(863) 210-2329</t>
-  </si>
-  <si>
-    <t>service@iceberghomeservices.com</t>
-  </si>
-  <si>
-    <t>https://iceberghomeservices.com</t>
+    <t>(863) 345-0493</t>
+  </si>
+  <si>
+    <t>(863) 223-1397</t>
+  </si>
+  <si>
+    <t>service@icebergcooling.com</t>
+  </si>
+  <si>
+    <t>https://icebergcooling.com</t>
   </si>
   <si>
     <t>4.7 (2,279 reviews)</t>
@@ -560,13 +553,16 @@
     <t>CAC1814697</t>
   </si>
   <si>
-    <t>(407) 633-4710</t>
-  </si>
-  <si>
-    <t>info@rainaldi.com</t>
-  </si>
-  <si>
-    <t>https://rainaldi.com</t>
+    <t>(407) 282-2900</t>
+  </si>
+  <si>
+    <t>(407) 413-9795</t>
+  </si>
+  <si>
+    <t>info@rainaldihomeservices.com</t>
+  </si>
+  <si>
+    <t>https://rainaldihomeservices.com</t>
   </si>
   <si>
     <t>4.8 (5,972 reviews)</t>
@@ -593,13 +589,16 @@
     <t>CAC057997</t>
   </si>
   <si>
-    <t>(407) 892-0690</t>
-  </si>
-  <si>
-    <t>info@franksair.com</t>
-  </si>
-  <si>
-    <t>https://franksair.com</t>
+    <t>(407) 490-2070</t>
+  </si>
+  <si>
+    <t>(407) 870-7755</t>
+  </si>
+  <si>
+    <t>info@franksac.com</t>
+  </si>
+  <si>
+    <t>https://franksac.com</t>
   </si>
   <si>
     <t>4.9 (2,679 reviews)</t>
@@ -623,7 +622,10 @@
     <t>CAC1816543 / CFC057530</t>
   </si>
   <si>
-    <t>(407) 993-1874</t>
+    <t>(407) 499-8006</t>
+  </si>
+  <si>
+    <t>(407) 857-0110</t>
   </si>
   <si>
     <t>info@acesolvesitall.com</t>
@@ -653,13 +655,13 @@
     <t>CAC1813476</t>
   </si>
   <si>
-    <t>(321) 290-9625</t>
-  </si>
-  <si>
-    <t>contact@americanairfl.com</t>
-  </si>
-  <si>
-    <t>https://americanairfl.com</t>
+    <t>(407) 603-4410</t>
+  </si>
+  <si>
+    <t>contact@americanairandheat.com</t>
+  </si>
+  <si>
+    <t>https://americanairandheat.com</t>
   </si>
   <si>
     <t>4.9 (10,285 reviews)</t>
@@ -686,7 +688,10 @@
     <t>CAC021115 / CFC057524</t>
   </si>
   <si>
-    <t>(407) 598-7733</t>
+    <t>(844) 909-3003</t>
+  </si>
+  <si>
+    <t>(888) 831-2665</t>
   </si>
   <si>
     <t>customercare@delair.com</t>
@@ -713,7 +718,10 @@
     <t>CAC1818012 / CFC057283</t>
   </si>
   <si>
-    <t>(407) 900-1175</t>
+    <t>(407) 204-0430</t>
+  </si>
+  <si>
+    <t>(407) 490-1361</t>
   </si>
   <si>
     <t>info@frankgayservices.com</t>
@@ -746,7 +754,7 @@
     <t>CAC1816914</t>
   </si>
   <si>
-    <t>(321) 290-9943</t>
+    <t>(321) 637-0170</t>
   </si>
   <si>
     <t>info@dittmerairandheat.com</t>
@@ -773,8 +781,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1004,6 +1012,15 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1022,36 +1039,19 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1089,7 +1089,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1123,7 +1123,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1158,10 +1157,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1334,1225 +1332,1225 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" customWidth="1"/>
-    <col min="3" max="3" width="41.85546875" customWidth="1"/>
-    <col min="4" max="4" width="35.5703125" customWidth="1"/>
-    <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="61.28515625" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.7109375" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" customWidth="1"/>
     <col min="8" max="9" width="18.7109375" customWidth="1"/>
     <col min="10" max="10" width="26.7109375" customWidth="1"/>
     <col min="11" max="11" width="24.7109375" customWidth="1"/>
     <col min="12" max="12" width="18.7109375" customWidth="1"/>
     <col min="13" max="13" width="22.7109375" customWidth="1"/>
-    <col min="14" max="14" width="121.7109375" customWidth="1"/>
-    <col min="15" max="15" width="93.85546875" customWidth="1"/>
+    <col min="14" max="14" width="44.7109375" customWidth="1"/>
+    <col min="15" max="15" width="30.7109375" customWidth="1"/>
     <col min="16" max="16" width="24.7109375" customWidth="1"/>
     <col min="17" max="17" width="18.7109375" customWidth="1"/>
     <col min="18" max="18" width="16.7109375" customWidth="1"/>
-    <col min="19" max="19" width="127.28515625" customWidth="1"/>
+    <col min="19" max="19" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:19" ht="32" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:19">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8" t="s">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8" t="s">
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="8"/>
+      <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:19" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="9">
+    <row r="4" spans="1:19">
+      <c r="A4" s="3">
         <f>COUNTA(C7:C200)</f>
-        <v>20</v>
-      </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3">
         <f>COUNTIF(B7:B200, "A*")</f>
-        <v>11</v>
-      </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3">
         <f>COUNTIF(A7:A200, "Demo Booked")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9">
+      <c r="F4" s="3"/>
+      <c r="G4" s="3">
         <f>COUNTIF(A7:A200, "&lt;&gt;Not Contacted") - COUNTBLANK(A7:A200)</f>
-        <v>3</v>
-      </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3">
         <f>COUNTIF(A7:A200, "Gatekeeper*") + COUNTIF(A7:A200, "Follow-up")</f>
-        <v>2</v>
-      </c>
-      <c r="J4" s="9"/>
+        <v>0</v>
+      </c>
+      <c r="J4" s="3"/>
     </row>
-    <row r="6" spans="1:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:19" ht="28" customHeight="1">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="N6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="O6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="P6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="Q6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="R6" s="1" t="s">
+      <c r="R6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="S6" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:19" ht="22" customHeight="1">
+      <c r="A7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="I7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="J7" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="K7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="L7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="M7" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2" t="s">
+      <c r="N7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="S7" s="2" t="s">
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5" t="s">
         <v>39</v>
       </c>
+      <c r="S7" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="8" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="4" t="s">
+    <row r="8" spans="1:19" ht="22" customHeight="1">
+      <c r="A8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="4" t="s">
+      <c r="F8" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="G8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="H8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="I8" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M8" s="4" t="s">
+      <c r="L8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M8" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="N8" s="4" t="s">
+      <c r="N8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="O8" s="4" t="s">
+      <c r="O8" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4" t="s">
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="S8" s="4" t="s">
+      <c r="S8" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:19" ht="22" customHeight="1">
+      <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="L9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M9" s="2" t="s">
+      <c r="L9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N9" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2" t="s">
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="S9" s="2" t="s">
+      <c r="S9" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:19" ht="22" customHeight="1">
+      <c r="A10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="I10" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="J10" s="4" t="s">
+      <c r="I10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="J10" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M10" s="4" t="s">
+      <c r="K10" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="4" t="s">
+      <c r="L10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M10" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4" t="s">
+      <c r="N10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="S10" s="4" t="s">
-        <v>73</v>
+      <c r="S10" s="7" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:19" ht="22" customHeight="1">
+      <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="C11" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="E11" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="F11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="G11" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="H11" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="I11" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="J11" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M11" s="2" t="s">
+      <c r="K11" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="L11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M11" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2" t="s">
+      <c r="N11" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="S11" s="2" t="s">
+      <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5" t="s">
         <v>85</v>
       </c>
+      <c r="S11" s="5" t="s">
+        <v>86</v>
+      </c>
     </row>
-    <row r="12" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:19" ht="22" customHeight="1">
+      <c r="A12" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G12" s="4" t="s">
+      <c r="F12" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="G12" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="I12" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="J12" s="4" t="s">
+      <c r="H12" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="I12" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="L12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M12" s="4" t="s">
+      <c r="K12" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="L12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M12" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4" t="s">
+      <c r="N12" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="S12" s="4" t="s">
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7" t="s">
         <v>95</v>
       </c>
+      <c r="S12" s="7" t="s">
+        <v>96</v>
+      </c>
     </row>
-    <row r="13" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:19" ht="22" customHeight="1">
+      <c r="A13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="C13" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="D13" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G13" s="2" t="s">
+      <c r="F13" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="G13" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J13" s="2" t="s">
+      <c r="H13" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="I13" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J13" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="L13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M13" s="2" t="s">
+      <c r="K13" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="L13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M13" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2" t="s">
+      <c r="N13" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="S13" s="2" t="s">
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5" t="s">
         <v>106</v>
       </c>
+      <c r="S13" s="5" t="s">
+        <v>107</v>
+      </c>
     </row>
-    <row r="14" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:19" ht="22" customHeight="1">
+      <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="G14" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I14" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="J14" s="4" t="s">
+      <c r="H14" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="I14" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="L14" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M14" s="4" t="s">
+      <c r="J14" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="N14" s="4" t="s">
+      <c r="K14" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4" t="s">
+      <c r="L14" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M14" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="S14" s="4" t="s">
+      <c r="N14" s="7" t="s">
         <v>116</v>
       </c>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="S14" s="7" t="s">
+        <v>118</v>
+      </c>
     </row>
-    <row r="15" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B15" s="2" t="s">
+    <row r="15" spans="1:19" ht="22" customHeight="1">
+      <c r="A15" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="C15" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G15" s="2" t="s">
+      <c r="E15" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="F15" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="J15" s="2" t="s">
+      <c r="G15" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="H15" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="L15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M15" s="2" t="s">
+      <c r="I15" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="J15" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="N15" s="2" t="s">
+      <c r="K15" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="O15" s="2" t="s">
+      <c r="L15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M15" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2" t="s">
+      <c r="N15" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="S15" s="2" t="s">
+      <c r="O15" s="5" t="s">
         <v>129</v>
       </c>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="S15" s="5" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:19" ht="22" customHeight="1">
+      <c r="A16" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="C16" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="H16" s="4" t="s">
+      <c r="F16" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="I16" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="J16" s="4" t="s">
+      <c r="G16" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="H16" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="L16" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M16" s="4" t="s">
+      <c r="I16" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="J16" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="S16" s="4" t="s">
+      <c r="K16" s="7" t="s">
         <v>138</v>
       </c>
+      <c r="L16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="S16" s="7" t="s">
+        <v>141</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:19" ht="22" customHeight="1">
+      <c r="A17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="C17" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="F17" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="G17" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="H17" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="L17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M17" s="2" t="s">
+      <c r="I17" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="N17" s="2" t="s">
+      <c r="J17" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2" t="s">
+      <c r="K17" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="S17" s="2" t="s">
+      <c r="L17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M17" s="5" t="s">
         <v>149</v>
       </c>
+      <c r="N17" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="S17" s="5" t="s">
+        <v>152</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:19" ht="22" customHeight="1">
+      <c r="A18" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E18" s="4" t="s">
+      <c r="B18" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="S18" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="22" customHeight="1">
+      <c r="A19" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="L18" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="N18" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>161</v>
+      <c r="C19" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M19" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="S19" s="5" t="s">
+        <v>175</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="20" spans="1:19" ht="22" customHeight="1">
+      <c r="A20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="S19" s="2" t="s">
-        <v>171</v>
+      <c r="B20" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="S20" s="7" t="s">
+        <v>186</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+    <row r="21" spans="1:19" ht="22" customHeight="1">
+      <c r="A21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="B21" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E21" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="L21" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M21" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="N21" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="S21" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="22" customHeight="1">
+      <c r="A22" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="S22" s="7" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="22" customHeight="1">
+      <c r="A23" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="L20" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="N20" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="O20" s="4"/>
-      <c r="P20" s="4"/>
-      <c r="Q20" s="4"/>
-      <c r="R20" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="S20" s="4" t="s">
-        <v>181</v>
+      <c r="F23" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="N23" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="O23" s="5"/>
+      <c r="P23" s="5"/>
+      <c r="Q23" s="5"/>
+      <c r="R23" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="S23" s="5" t="s">
+        <v>219</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+    <row r="24" spans="1:19" ht="22" customHeight="1">
+      <c r="A24" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="B24" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="O24" s="7"/>
+      <c r="P24" s="7"/>
+      <c r="Q24" s="7"/>
+      <c r="R24" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="S24" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="22" customHeight="1">
+      <c r="A25" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="N25" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="S25" s="5" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="22" customHeight="1">
+      <c r="A26" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="S21" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="L22" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="N22" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="S22" s="4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="23" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="S23" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="N24" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="O24" s="4"/>
-      <c r="P24" s="4"/>
-      <c r="Q24" s="4"/>
-      <c r="R24" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="S24" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="S25" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="J26" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="K26" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="L26" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M26" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="N26" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="O26" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="P26" s="4"/>
-      <c r="Q26" s="4"/>
-      <c r="R26" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="S26" s="4" t="s">
+      <c r="E26" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F26" s="7" t="s">
         <v>244</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="N26" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="O26" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="7"/>
+      <c r="R26" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="S26" s="7" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -2570,37 +2568,37 @@
     <mergeCell ref="I4:J4"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A7:A200" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A7:A200">
       <formula1>"Not Contacted,Called - No Answer,SMS Sent,Gatekeeper / Callback,Follow-up,Demo Booked,Closed Won,Disqualified"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B200" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B200">
       <formula1>"A - High (Sweet Spot / Fast Conversion),B - Medium (Scale / Multi-Tech),C - Disqualified / Do Not Call"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7:L200" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7:L200">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="K7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="K8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="K9" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="K10" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="K11" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="K12" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="K13" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="K14" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="K15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="K16" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="K17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="K18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="K19" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="K20" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="K21" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="K22" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="K23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="K24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="K25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="K26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="K7" r:id="rId1"/>
+    <hyperlink ref="K8" r:id="rId2"/>
+    <hyperlink ref="K9" r:id="rId3"/>
+    <hyperlink ref="K10" r:id="rId4"/>
+    <hyperlink ref="K11" r:id="rId5"/>
+    <hyperlink ref="K12" r:id="rId6"/>
+    <hyperlink ref="K13" r:id="rId7"/>
+    <hyperlink ref="K14" r:id="rId8"/>
+    <hyperlink ref="K15" r:id="rId9"/>
+    <hyperlink ref="K16" r:id="rId10"/>
+    <hyperlink ref="K17" r:id="rId11"/>
+    <hyperlink ref="K18" r:id="rId12"/>
+    <hyperlink ref="K19" r:id="rId13"/>
+    <hyperlink ref="K20" r:id="rId14"/>
+    <hyperlink ref="K21" r:id="rId15"/>
+    <hyperlink ref="K22" r:id="rId16"/>
+    <hyperlink ref="K23" r:id="rId17"/>
+    <hyperlink ref="K24" r:id="rId18"/>
+    <hyperlink ref="K25" r:id="rId19"/>
+    <hyperlink ref="K26" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>